<commit_message>
Rebase real-only governance and evidence audit onto current main
</commit_message>
<xml_diff>
--- a/03_Private_Equity/instances/public_home_depot_2023.xlsx
+++ b/03_Private_Equity/instances/public_home_depot_2023.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="312">
   <si>
     <t xml:space="preserve">[TARGET] — LBO Underwriting Model</t>
   </si>
@@ -47,13 +47,13 @@
     <t xml:space="preserve">Target / transaction:</t>
   </si>
   <si>
-    <t xml:space="preserve">The Home Depot FY2023 public-company operating case</t>
+    <t xml:space="preserve">[Name]</t>
   </si>
   <si>
     <t xml:space="preserve">Sponsor / principal:</t>
   </si>
   <si>
-    <t xml:space="preserve">Benchmark Sponsor</t>
+    <t xml:space="preserve">[Fund / merchant bank]</t>
   </si>
   <si>
     <t xml:space="preserve">Entry / close date:</t>
@@ -942,15 +942,6 @@
   </si>
   <si>
     <t xml:space="preserve">Immutable curated observation package with SHA-256 digest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retained modeler assumption from pe-reference-buyout.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">repo://standards/benchmark_cases/pe-reference-buyout.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not an external observation; retained for sensitivity and transaction-structure completeness</t>
   </si>
   <si>
     <t xml:space="preserve">Refresh Log</t>
@@ -1114,14 +1105,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -1198,7 +1189,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1227,7 +1218,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1267,11 +1258,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1279,11 +1270,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1291,7 +1282,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1303,15 +1294,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1446,34 +1433,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1619,7 +1606,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:F17"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="36"/>
@@ -1656,7 +1643,7 @@
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1664,7 +1651,7 @@
       <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1672,7 +1659,7 @@
       <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1680,7 +1667,7 @@
       <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1688,7 +1675,7 @@
       <c r="B10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1760,7 +1747,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:E9"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
@@ -1827,7 +1814,7 @@
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">'Sources &amp; Uses'!F8</f>
-        <v>121817.03997</v>
+        <v>109904.2779</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>127</v>
@@ -1842,7 +1829,7 @@
       </c>
       <c r="C8" s="19" t="n">
         <f aca="false">C7*(1+Assumptions!E31)^Assumptions!E29</f>
-        <v>178989.197060589</v>
+        <v>161485.4412789</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>127</v>
@@ -1886,7 +1873,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:J15"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
@@ -1976,35 +1963,35 @@
       <c r="B6" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="26" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>10</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="26" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>10</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="26" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>10</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="26" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>10</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="26" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>10</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="26" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>10</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="26" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>10</v>
       </c>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="26" t="n">
         <f aca="false">INDEX(C6:I6,1,Assumptions!E29)</f>
         <v>10</v>
       </c>
@@ -2052,35 +2039,35 @@
       </c>
       <c r="C8" s="19" t="n">
         <f aca="false">'Debt Schedule'!D28</f>
-        <v>124407.000235313</v>
+        <v>124691.68021125</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">'Debt Schedule'!E28</f>
-        <v>119998.7349601</v>
+        <v>120595.047125562</v>
       </c>
       <c r="E8" s="19" t="n">
         <f aca="false">'Debt Schedule'!F28</f>
-        <v>115204.363395756</v>
+        <v>116141.578836387</v>
       </c>
       <c r="F8" s="19" t="n">
         <f aca="false">'Debt Schedule'!G28</f>
-        <v>110013.616979535</v>
+        <v>111323.384621118</v>
       </c>
       <c r="G8" s="19" t="n">
         <f aca="false">'Debt Schedule'!H28</f>
-        <v>104415.190086469</v>
+        <v>106131.715854733</v>
       </c>
       <c r="H8" s="19" t="n">
         <f aca="false">'Debt Schedule'!I28</f>
-        <v>98395.916190782</v>
+        <v>100556.162874162</v>
       </c>
       <c r="I8" s="19" t="n">
         <f aca="false">'Debt Schedule'!J28</f>
-        <v>91940.6238682786</v>
+        <v>94584.5269144406</v>
       </c>
       <c r="J8" s="19" t="n">
         <f aca="false">INDEX(C8:I8,1,Assumptions!E29)</f>
-        <v>104415.190086469</v>
+        <v>106131.715854733</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2089,35 +2076,35 @@
       </c>
       <c r="C9" s="19" t="n">
         <f aca="false">MAX(0,C7-C8)</f>
-        <v>109573.509164687</v>
+        <v>109288.82918875</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">MAX(0,D7-D8)</f>
-        <v>114144.6722629</v>
+        <v>113548.360097438</v>
       </c>
       <c r="E9" s="19" t="n">
         <f aca="false">MAX(0,E7-E8)</f>
-        <v>118881.585322404</v>
+        <v>117944.369881773</v>
       </c>
       <c r="F9" s="19" t="n">
         <f aca="false">MAX(0,F7-F8)</f>
-        <v>123807.591677574</v>
+        <v>122497.824035991</v>
       </c>
       <c r="G9" s="19" t="n">
         <f aca="false">MAX(0,G7-G8)</f>
-        <v>128946.485559407</v>
+        <v>127229.959791143</v>
       </c>
       <c r="H9" s="19" t="n">
         <f aca="false">MAX(0,H7-H8)</f>
-        <v>134323.359336743</v>
+        <v>132163.112653363</v>
       </c>
       <c r="I9" s="19" t="n">
         <f aca="false">MAX(0,I7-I8)</f>
-        <v>139964.770039915</v>
+        <v>137320.866993753</v>
       </c>
       <c r="J9" s="19" t="n">
         <f aca="false">INDEX(C9:I9,1,Assumptions!E29)</f>
-        <v>128946.485559407</v>
+        <v>127229.959791143</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2126,35 +2113,35 @@
       </c>
       <c r="C10" s="19" t="n">
         <f aca="false">'Management Equity'!$C$7*(1+Assumptions!$E$31)^1</f>
-        <v>131562.4031676</v>
+        <v>118696.620132</v>
       </c>
       <c r="D10" s="19" t="n">
         <f aca="false">'Management Equity'!$C$7*(1+Assumptions!$E$31)^2</f>
-        <v>142087.395421008</v>
+        <v>128192.34974256</v>
       </c>
       <c r="E10" s="19" t="n">
         <f aca="false">'Management Equity'!$C$7*(1+Assumptions!$E$31)^3</f>
-        <v>153454.387054689</v>
+        <v>138447.737721965</v>
       </c>
       <c r="F10" s="19" t="n">
         <f aca="false">'Management Equity'!$C$7*(1+Assumptions!$E$31)^4</f>
-        <v>165730.738019064</v>
+        <v>149523.556739722</v>
       </c>
       <c r="G10" s="19" t="n">
         <f aca="false">'Management Equity'!$C$7*(1+Assumptions!$E$31)^5</f>
-        <v>178989.197060589</v>
+        <v>161485.4412789</v>
       </c>
       <c r="H10" s="19" t="n">
         <f aca="false">'Management Equity'!$C$7*(1+Assumptions!$E$31)^6</f>
-        <v>193308.332825436</v>
+        <v>174404.276581212</v>
       </c>
       <c r="I10" s="19" t="n">
         <f aca="false">'Management Equity'!$C$7*(1+Assumptions!$E$31)^7</f>
-        <v>208772.999451471</v>
+        <v>188356.618707709</v>
       </c>
       <c r="J10" s="19" t="n">
         <f aca="false">INDEX(C10:I10,1,Assumptions!E29)</f>
-        <v>178989.197060589</v>
+        <v>161485.4412789</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2200,35 +2187,35 @@
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">MIN(C9,C9*Assumptions!$E$30+C11*Assumptions!$E$32)</f>
-        <v>10957.3509164688</v>
+        <v>10928.882918875</v>
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">MIN(D9,D9*Assumptions!$E$30+D11*Assumptions!$E$32)</f>
-        <v>11414.46722629</v>
+        <v>11354.8360097438</v>
       </c>
       <c r="E12" s="19" t="n">
         <f aca="false">MIN(E9,E9*Assumptions!$E$30+E11*Assumptions!$E$32)</f>
-        <v>11888.1585322404</v>
+        <v>11794.4369881773</v>
       </c>
       <c r="F12" s="19" t="n">
         <f aca="false">MIN(F9,F9*Assumptions!$E$30+F11*Assumptions!$E$32)</f>
-        <v>12380.7591677574</v>
+        <v>12249.7824035991</v>
       </c>
       <c r="G12" s="19" t="n">
         <f aca="false">MIN(G9,G9*Assumptions!$E$30+G11*Assumptions!$E$32)</f>
-        <v>12894.6485559407</v>
+        <v>12722.9959791143</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">MIN(H9,H9*Assumptions!$E$30+H11*Assumptions!$E$32)</f>
-        <v>13432.3359336743</v>
+        <v>13216.3112653363</v>
       </c>
       <c r="I12" s="19" t="n">
         <f aca="false">MIN(I9,I9*Assumptions!$E$30+I11*Assumptions!$E$32)</f>
-        <v>13996.4770039915</v>
+        <v>13732.0866993753</v>
       </c>
       <c r="J12" s="19" t="n">
         <f aca="false">INDEX(C12:I12,1,Assumptions!E29)</f>
-        <v>12894.6485559407</v>
+        <v>12722.9959791143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2237,72 +2224,72 @@
       </c>
       <c r="C13" s="19" t="n">
         <f aca="false">MAX(0,C9-C12)</f>
-        <v>98616.1582482187</v>
+        <v>98359.946269875</v>
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">MAX(0,D9-D12)</f>
-        <v>102730.20503661</v>
+        <v>102193.524087694</v>
       </c>
       <c r="E13" s="19" t="n">
         <f aca="false">MAX(0,E9-E12)</f>
-        <v>106993.426790163</v>
+        <v>106149.932893595</v>
       </c>
       <c r="F13" s="19" t="n">
         <f aca="false">MAX(0,F9-F12)</f>
-        <v>111426.832509817</v>
+        <v>110248.041632392</v>
       </c>
       <c r="G13" s="19" t="n">
         <f aca="false">MAX(0,G9-G12)</f>
-        <v>116051.837003466</v>
+        <v>114506.963812029</v>
       </c>
       <c r="H13" s="19" t="n">
         <f aca="false">MAX(0,H9-H12)</f>
-        <v>120891.023403069</v>
+        <v>118946.801388027</v>
       </c>
       <c r="I13" s="19" t="n">
         <f aca="false">MAX(0,I9-I12)</f>
-        <v>125968.293035924</v>
+        <v>123588.780294378</v>
       </c>
       <c r="J13" s="19" t="n">
         <f aca="false">INDEX(C13:I13,1,Assumptions!E29)</f>
-        <v>116051.837003466</v>
+        <v>114506.963812029</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="26" t="n">
         <f aca="false">IFERROR(C13/'Sources &amp; Uses'!$F$8,0)</f>
-        <v>0.80954321556742</v>
-      </c>
-      <c r="D14" s="27" t="n">
+        <v>0.894960124840372</v>
+      </c>
+      <c r="D14" s="26" t="n">
         <f aca="false">IFERROR(D13/'Sources &amp; Uses'!$F$8,0)</f>
-        <v>0.843315558003296</v>
-      </c>
-      <c r="E14" s="27" t="n">
+        <v>0.929841185806055</v>
+      </c>
+      <c r="E14" s="26" t="n">
         <f aca="false">IFERROR(E13/'Sources &amp; Uses'!$F$8,0)</f>
-        <v>0.878312482527179</v>
-      </c>
-      <c r="F14" s="27" t="n">
+        <v>0.965839864670048</v>
+      </c>
+      <c r="F14" s="26" t="n">
         <f aca="false">IFERROR(F13/'Sources &amp; Uses'!$F$8,0)</f>
-        <v>0.914706452703645</v>
-      </c>
-      <c r="G14" s="27" t="n">
+        <v>1.00312784669497</v>
+      </c>
+      <c r="G14" s="26" t="n">
         <f aca="false">IFERROR(G13/'Sources &amp; Uses'!$F$8,0)</f>
-        <v>0.952673263379626</v>
-      </c>
-      <c r="H14" s="27" t="n">
+        <v>1.04187904238102</v>
+      </c>
+      <c r="H14" s="26" t="n">
         <f aca="false">IFERROR(H13/'Sources &amp; Uses'!$F$8,0)</f>
-        <v>0.992398300211864</v>
-      </c>
-      <c r="I14" s="27" t="n">
+        <v>1.0822763559418</v>
+      </c>
+      <c r="I14" s="26" t="n">
         <f aca="false">IFERROR(I13/'Sources &amp; Uses'!$F$8,0)</f>
-        <v>1.03407776996507</v>
-      </c>
-      <c r="J14" s="27" t="n">
+        <v>1.12451291847647</v>
+      </c>
+      <c r="J14" s="26" t="n">
         <f aca="false">INDEX(C14:I14,1,Assumptions!E29)</f>
-        <v>0.952673263379626</v>
+        <v>1.04187904238102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2311,35 +2298,35 @@
       </c>
       <c r="C15" s="24" t="n">
         <f aca="false">IFERROR((C13/'Sources &amp; Uses'!$F$8)^(1/1)-1,0)</f>
-        <v>-0.19045678443258</v>
+        <v>-0.105039875159628</v>
       </c>
       <c r="D15" s="24" t="n">
         <f aca="false">IFERROR((D13/'Sources &amp; Uses'!$F$8)^(1/2)-1,0)</f>
-        <v>-0.0816778571746756</v>
+        <v>-0.0357172687400985</v>
       </c>
       <c r="E15" s="24" t="n">
         <f aca="false">IFERROR((E13/'Sources &amp; Uses'!$F$8)^(1/3)-1,0)</f>
-        <v>-0.0423289663639923</v>
+        <v>-0.0115188870758636</v>
       </c>
       <c r="F15" s="24" t="n">
         <f aca="false">IFERROR((F13/'Sources &amp; Uses'!$F$8)^(1/4)-1,0)</f>
-        <v>-0.0220414775936785</v>
+        <v>0.000781046147557918</v>
       </c>
       <c r="G15" s="24" t="n">
         <f aca="false">IFERROR((G13/'Sources &amp; Uses'!$F$8)^(1/5)-1,0)</f>
-        <v>-0.00964979595199322</v>
+        <v>0.00823892555745531</v>
       </c>
       <c r="H15" s="24" t="n">
         <f aca="false">IFERROR((H13/'Sources &amp; Uses'!$F$8)^(1/6)-1,0)</f>
-        <v>-0.0012709816130736</v>
+        <v>0.013264969325727</v>
       </c>
       <c r="I15" s="24" t="n">
         <f aca="false">IFERROR((I13/'Sources &amp; Uses'!$F$8)^(1/7)-1,0)</f>
-        <v>0.00479861752067445</v>
+        <v>0.0169055920708845</v>
       </c>
       <c r="J15" s="24" t="n">
         <f aca="false">INDEX(C15:I15,1,Assumptions!E29)</f>
-        <v>-0.00964979595199322</v>
+        <v>0.00823892555745531</v>
       </c>
     </row>
   </sheetData>
@@ -2362,7 +2349,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:G9"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28"/>
@@ -2383,145 +2370,145 @@
       <c r="B4" s="16" t="s">
         <v>263</v>
       </c>
-      <c r="C4" s="32" t="n">
+      <c r="C4" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="D4" s="32" t="n">
+      <c r="D4" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="32" t="n">
+      <c r="E4" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="F4" s="32" t="n">
+      <c r="F4" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="G4" s="32" t="n">
+      <c r="G4" s="31" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="27" t="n">
+      <c r="B5" s="26" t="n">
         <v>8</v>
       </c>
       <c r="C5" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*C$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B5+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0541733166544571</v>
+        <v>-0.0581698451093956</v>
       </c>
       <c r="D5" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*D$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B5+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.0170288187806811</v>
+        <v>0.0142785049827239</v>
       </c>
       <c r="E5" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*E$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B5+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.0725363268430281</v>
+        <v>0.0705019893213061</v>
       </c>
       <c r="F5" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*F$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B5+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.11847980385338</v>
+        <v>0.116918290461881</v>
       </c>
       <c r="G5" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*G$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B5+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.157919494431067</v>
+        <v>0.156697512238684</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="26" t="n">
         <v>9</v>
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*C$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B6+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.111668734051856</v>
+        <v>-0.115598250497523</v>
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*D$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B6+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0447948720398664</v>
+        <v>-0.0475674625286657</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*E$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B6+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.00733841598732021</v>
+        <v>0.00522777624550885</v>
       </c>
       <c r="F6" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*F$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B6+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.050489056388269</v>
+        <v>0.0488138280628094</v>
       </c>
       <c r="G6" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*G$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B6+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.0875312659985466</v>
+        <v>0.0861674986270506</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="26" t="n">
         <v>10</v>
       </c>
       <c r="C7" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*C$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B7+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.153024099676384</v>
+        <v>-0.156867181583465</v>
       </c>
       <c r="D7" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*D$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B7+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0892634828244395</v>
+        <v>-0.0920109213696565</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*E$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B7+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0395572074109225</v>
+        <v>-0.0416792723292913</v>
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*F$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B7+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.00158459847173531</v>
+        <v>-0.000127080994252737</v>
       </c>
       <c r="G7" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*G$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B7+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>0.0369023453948436</v>
+        <v>0.0354835513442162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="26" t="n">
         <v>11</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*C$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B8+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.184986901879388</v>
+        <v>-0.188745283917349</v>
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*D$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B8+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.123632455007017</v>
+        <v>-0.126341181246135</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*E$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B8+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.075801973047225</v>
+        <v>-0.0779125271120233</v>
       </c>
       <c r="F8" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*F$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B8+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0362127584522289</v>
+        <v>-0.0379313871921857</v>
       </c>
       <c r="G8" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*G$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B8+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0022278170537261</v>
+        <v>-0.00366716120520005</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="26" t="n">
         <v>12</v>
       </c>
       <c r="C9" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*C$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B9+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.210851123106239</v>
+        <v>-0.214531234724911</v>
       </c>
       <c r="D9" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*D$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B9+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.151443743085698</v>
+        <v>-0.154110663353755</v>
       </c>
       <c r="E9" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*E$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B9+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.105131148592559</v>
+        <v>-0.107221327103931</v>
       </c>
       <c r="F9" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*F$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B9+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0667982870633519</v>
+        <v>-0.0685109985418146</v>
       </c>
       <c r="G9" s="22" t="n">
         <f aca="false">IFERROR(((('Operating Model'!H8*G$4-'Debt Schedule'!G28)*(1-Assumptions!$E$30))/MAX(0.01,('Operating Model'!C8*$B9+Assumptions!$E$15+'Sources &amp; Uses'!C7+Assumptions!$E$16-'Sources &amp; Uses'!F6-'Sources &amp; Uses'!F7)))^(1/5)-1,0)</f>
-        <v>-0.0338918486296963</v>
+        <v>-0.0353358702552724</v>
       </c>
     </row>
   </sheetData>
@@ -2556,7 +2543,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:C13"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
@@ -2691,8 +2678,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:E12"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B2:E11"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
@@ -2724,115 +2711,101 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="32" t="s">
         <v>279</v>
       </c>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="32" t="s">
         <v>280</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="32" t="s">
         <v>281</v>
       </c>
-      <c r="E5" s="33" t="s">
+      <c r="E5" s="32" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="32" t="s">
         <v>283</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="32" t="s">
         <v>284</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="33" t="s">
+      <c r="E6" s="32" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="32" t="s">
         <v>286</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="32" t="s">
         <v>287</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="D7" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="32" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="32" t="s">
         <v>289</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="32" t="s">
         <v>290</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="33" t="s">
+      <c r="E8" s="32" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="32" t="s">
         <v>292</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="32" t="s">
         <v>293</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="33" t="s">
+      <c r="E9" s="32" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="33" t="s">
         <v>295</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="33" t="s">
         <v>296</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="34" t="s">
+      <c r="E10" s="33" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="33" t="s">
         <v>298</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="33" t="s">
         <v>299</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="34" t="s">
+      <c r="E11" s="33" t="s">
         <v>300</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="34" t="s">
-        <v>301</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>302</v>
-      </c>
-      <c r="D12" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -2855,7 +2828,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:G29"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
@@ -2868,7 +2841,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2881,232 +2854,232 @@
         <v>94</v>
       </c>
       <c r="C4" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="G4" s="16" t="s">
         <v>306</v>
       </c>
-      <c r="E4" s="16" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="34" t="s">
         <v>307</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="C5" s="34" t="s">
         <v>308</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="D5" s="34" t="s">
+        <v>299</v>
+      </c>
+      <c r="E5" s="34" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="35" t="s">
+      <c r="F5" s="34" t="s">
         <v>310</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="G5" s="34" t="s">
         <v>311</v>
       </c>
-      <c r="D5" s="35" t="s">
-        <v>299</v>
-      </c>
-      <c r="E5" s="35" t="s">
-        <v>312</v>
-      </c>
-      <c r="F5" s="35" t="s">
-        <v>313</v>
-      </c>
-      <c r="G5" s="35" t="s">
-        <v>314</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="35"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="35"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="35"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="35"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35"/>
-      <c r="G25" s="35"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="35"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35"/>
-      <c r="G26" s="35"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="35"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="35"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="35"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3128,7 +3101,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:F63"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
@@ -3885,7 +3858,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:I9"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
@@ -4035,7 +4008,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:J8"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
@@ -4192,7 +4165,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:F32"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
@@ -4375,14 +4348,14 @@
         <v>137</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="D13" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="26" t="n">
         <f aca="false">IF(Cover!$C$9="Downside",D13,C13)</f>
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>138</v>
@@ -4483,14 +4456,14 @@
         <v>144</v>
       </c>
       <c r="C19" s="25" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="D19" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="25" t="n">
         <v>3.5</v>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E19" s="26" t="n">
         <f aca="false">IF(Cover!$C$9="Downside",D19,C19)</f>
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>145</v>
@@ -4537,14 +4510,14 @@
         <v>149</v>
       </c>
       <c r="C22" s="25" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="D22" s="26" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D22" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="27" t="n">
+      <c r="E22" s="26" t="n">
         <f aca="false">IF(Cover!$C$9="Downside",D22,C22)</f>
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>145</v>
@@ -4608,13 +4581,13 @@
       <c r="B26" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C26" s="26" t="n">
+      <c r="C26" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="D26" s="26" t="n">
+      <c r="D26" s="25" t="n">
         <v>6.5</v>
       </c>
-      <c r="E26" s="27" t="n">
+      <c r="E26" s="26" t="n">
         <f aca="false">IF(Cover!$C$9="Downside",D26,C26)</f>
         <v>7</v>
       </c>
@@ -4626,13 +4599,13 @@
       <c r="B27" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C27" s="26" t="n">
+      <c r="C27" s="25" t="n">
         <v>1.75</v>
       </c>
-      <c r="D27" s="26" t="n">
+      <c r="D27" s="25" t="n">
         <v>1.5</v>
       </c>
-      <c r="E27" s="27" t="n">
+      <c r="E27" s="26" t="n">
         <f aca="false">IF(Cover!$C$9="Downside",D27,C27)</f>
         <v>1.75</v>
       </c>
@@ -4647,10 +4620,10 @@
       <c r="C28" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="D28" s="26" t="n">
+      <c r="D28" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="E28" s="27" t="n">
+      <c r="E28" s="26" t="n">
         <f aca="false">IF(Cover!$C$9="Downside",D28,C28)</f>
         <v>10</v>
       </c>
@@ -4662,13 +4635,13 @@
       <c r="B29" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C29" s="28" t="n">
+      <c r="C29" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="D29" s="28" t="n">
+      <c r="D29" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="E29" s="29" t="n">
+      <c r="E29" s="28" t="n">
         <f aca="false">IF(Cover!$C$9="Downside",D29,C29)</f>
         <v>5</v>
       </c>
@@ -4750,7 +4723,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:G10"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
@@ -4793,7 +4766,7 @@
       </c>
       <c r="C5" s="19" t="n">
         <f aca="false">Assumptions!E5*Assumptions!E6*Assumptions!E13</f>
-        <v>245262.7485</v>
+        <v>233583.57</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>169</v>
@@ -4815,7 +4788,7 @@
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">Assumptions!E5*Assumptions!E6*Assumptions!E19</f>
-        <v>99273.01725</v>
+        <v>93433.428</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4824,14 +4797,14 @@
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">C5*Assumptions!E14</f>
-        <v>4905.25497</v>
+        <v>4671.6714</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>173</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">Assumptions!E5*Assumptions!E6*Assumptions!E22</f>
-        <v>29197.94625</v>
+        <v>35037.5355</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4847,23 +4820,23 @@
       </c>
       <c r="F8" s="19" t="n">
         <f aca="false">C9-SUM(F5:F7)</f>
-        <v>121817.03997</v>
+        <v>109904.2779</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="29" t="s">
         <v>176</v>
       </c>
-      <c r="C9" s="31" t="n">
+      <c r="C9" s="30" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>250288.00347</v>
-      </c>
-      <c r="E9" s="30" t="s">
+        <v>238375.2414</v>
+      </c>
+      <c r="E9" s="29" t="s">
         <v>177</v>
       </c>
-      <c r="F9" s="31" t="n">
+      <c r="F9" s="30" t="n">
         <f aca="false">SUM(F5:F8)</f>
-        <v>250288.00347</v>
+        <v>238375.2414</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4895,7 +4868,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:J19"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="36"/>
@@ -5051,38 +5024,38 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="29" t="s">
         <v>192</v>
       </c>
-      <c r="C8" s="31" t="n">
+      <c r="C8" s="30" t="n">
         <f aca="false">C5*C7</f>
         <v>23358.357</v>
       </c>
-      <c r="D8" s="31" t="n">
+      <c r="D8" s="30" t="n">
         <f aca="false">D5*D7</f>
         <v>23398.05094</v>
       </c>
-      <c r="E8" s="31" t="n">
+      <c r="E8" s="30" t="n">
         <f aca="false">E5*E7</f>
         <v>23414.3407223</v>
       </c>
-      <c r="F8" s="31" t="n">
+      <c r="F8" s="30" t="n">
         <f aca="false">F5*F7</f>
         <v>23408.594871816</v>
       </c>
-      <c r="G8" s="31" t="n">
+      <c r="G8" s="30" t="n">
         <f aca="false">G5*G7</f>
         <v>23382.120865711</v>
       </c>
-      <c r="H8" s="31" t="n">
+      <c r="H8" s="30" t="n">
         <f aca="false">H5*H7</f>
         <v>23336.1675645876</v>
       </c>
-      <c r="I8" s="31" t="n">
+      <c r="I8" s="30" t="n">
         <f aca="false">I5*I7</f>
         <v>23271.9275527525</v>
       </c>
-      <c r="J8" s="31" t="n">
+      <c r="J8" s="30" t="n">
         <f aca="false">J5*J7</f>
         <v>23190.5393908194</v>
       </c>
@@ -5167,31 +5140,31 @@
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">'Debt Schedule'!D7</f>
-        <v>11649.98055375</v>
+        <v>11795.970285</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">'Debt Schedule'!E7</f>
-        <v>11330.5966181139</v>
+        <v>11505.1319040023</v>
       </c>
       <c r="F11" s="19" t="n">
         <f aca="false">'Debt Schedule'!F7</f>
-        <v>10959.8723196736</v>
+        <v>11165.6387475201</v>
       </c>
       <c r="G11" s="19" t="n">
         <f aca="false">'Debt Schedule'!G7</f>
-        <v>10553.3547778563</v>
+        <v>10793.1016843274</v>
       </c>
       <c r="H11" s="19" t="n">
         <f aca="false">'Debt Schedule'!H7</f>
-        <v>10111.1115087954</v>
+        <v>10387.7988438072</v>
       </c>
       <c r="I11" s="19" t="n">
         <f aca="false">'Debt Schedule'!I7</f>
-        <v>9632.14718477652</v>
+        <v>9948.97027364607</v>
       </c>
       <c r="J11" s="19" t="n">
         <f aca="false">'Debt Schedule'!J7</f>
-        <v>9115.24027114113</v>
+        <v>9475.64867775454</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5200,31 +5173,31 @@
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">D10-D11</f>
-        <v>8045.84713625</v>
+        <v>7899.857405</v>
       </c>
       <c r="E12" s="19" t="n">
         <f aca="false">E10-E11</f>
-        <v>8492.58755168613</v>
+        <v>8318.05226579765</v>
       </c>
       <c r="F12" s="19" t="n">
         <f aca="false">F10-F11</f>
-        <v>8965.30069621743</v>
+        <v>8759.5342683709</v>
       </c>
       <c r="G12" s="19" t="n">
         <f aca="false">G10-G11</f>
-        <v>9449.84688760741</v>
+        <v>9210.09998113632</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">H10-H11</f>
-        <v>9947.50443155237</v>
+        <v>9670.81709654059</v>
       </c>
       <c r="I12" s="19" t="n">
         <f aca="false">I10-I11</f>
-        <v>10460.5552924634</v>
+        <v>10143.7322035938</v>
       </c>
       <c r="J12" s="19" t="n">
         <f aca="false">J10-J11</f>
-        <v>10991.450796431</v>
+        <v>10631.0423898176</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5233,31 +5206,31 @@
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">MAX(0,D12*Assumptions!$E$12)</f>
-        <v>2011.4617840625</v>
+        <v>1974.96435125</v>
       </c>
       <c r="E13" s="19" t="n">
         <f aca="false">MAX(0,E12*Assumptions!$E$12)</f>
-        <v>2123.14688792153</v>
+        <v>2079.51306644941</v>
       </c>
       <c r="F13" s="19" t="n">
         <f aca="false">MAX(0,F12*Assumptions!$E$12)</f>
-        <v>2241.32517405436</v>
+        <v>2189.88356709272</v>
       </c>
       <c r="G13" s="19" t="n">
         <f aca="false">MAX(0,G12*Assumptions!$E$12)</f>
-        <v>2362.46172190185</v>
+        <v>2302.52499528408</v>
       </c>
       <c r="H13" s="19" t="n">
         <f aca="false">MAX(0,H12*Assumptions!$E$12)</f>
-        <v>2486.87610788809</v>
+        <v>2417.70427413515</v>
       </c>
       <c r="I13" s="19" t="n">
         <f aca="false">MAX(0,I12*Assumptions!$E$12)</f>
-        <v>2615.13882311584</v>
+        <v>2535.93305089845</v>
       </c>
       <c r="J13" s="19" t="n">
         <f aca="false">MAX(0,J12*Assumptions!$E$12)</f>
-        <v>2747.86269910775</v>
+        <v>2657.7605974544</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5266,31 +5239,31 @@
       </c>
       <c r="D14" s="19" t="n">
         <f aca="false">D12-D13</f>
-        <v>6034.3853521875</v>
+        <v>5924.89305375</v>
       </c>
       <c r="E14" s="19" t="n">
         <f aca="false">E12-E13</f>
-        <v>6369.4406637646</v>
+        <v>6238.53919934824</v>
       </c>
       <c r="F14" s="19" t="n">
         <f aca="false">F12-F13</f>
-        <v>6723.97552216307</v>
+        <v>6569.65070127817</v>
       </c>
       <c r="G14" s="19" t="n">
         <f aca="false">G12-G13</f>
-        <v>7087.38516570556</v>
+        <v>6907.57498585224</v>
       </c>
       <c r="H14" s="19" t="n">
         <f aca="false">H12-H13</f>
-        <v>7460.62832366428</v>
+        <v>7253.11282240544</v>
       </c>
       <c r="I14" s="19" t="n">
         <f aca="false">I12-I13</f>
-        <v>7845.41646934752</v>
+        <v>7607.79915269535</v>
       </c>
       <c r="J14" s="19" t="n">
         <f aca="false">J12-J13</f>
-        <v>8243.58809732325</v>
+        <v>7973.28179236319</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5397,71 +5370,71 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="30" t="s">
+      <c r="B18" s="29" t="s">
         <v>202</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31" t="n">
+      <c r="C18" s="30"/>
+      <c r="D18" s="30" t="n">
         <f aca="false">D14+D9-D15-D17</f>
-        <v>4919.9016521875</v>
-      </c>
-      <c r="E18" s="31" t="n">
+        <v>4810.40935375</v>
+      </c>
+      <c r="E18" s="30" t="n">
         <f aca="false">E14+E9-E15-E17</f>
-        <v>5288.3914747646</v>
-      </c>
-      <c r="F18" s="31" t="n">
+        <v>5157.49001034824</v>
+      </c>
+      <c r="F18" s="30" t="n">
         <f aca="false">F14+F9-F15-F17</f>
-        <v>5675.35780883307</v>
-      </c>
-      <c r="G18" s="31" t="n">
+        <v>5521.03298794817</v>
+      </c>
+      <c r="G18" s="30" t="n">
         <f aca="false">G14+G9-G15-G17</f>
-        <v>6070.22598377546</v>
-      </c>
-      <c r="H18" s="31" t="n">
+        <v>5890.41580392214</v>
+      </c>
+      <c r="H18" s="30" t="n">
         <f aca="false">H14+H9-H15-H17</f>
-        <v>6473.98391719208</v>
-      </c>
-      <c r="I18" s="31" t="n">
+        <v>6266.46841593325</v>
+      </c>
+      <c r="I18" s="30" t="n">
         <f aca="false">I14+I9-I15-I17</f>
-        <v>6888.37139506949</v>
-      </c>
-      <c r="J18" s="31" t="n">
+        <v>6650.75407841732</v>
+      </c>
+      <c r="J18" s="30" t="n">
         <f aca="false">J14+J9-J15-J17</f>
-        <v>7315.25437527356</v>
+        <v>7044.9480703135</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31" t="n">
+      <c r="C19" s="30"/>
+      <c r="D19" s="30" t="n">
         <f aca="false">D8-D13-D15-D17</f>
-        <v>16569.8822059375</v>
-      </c>
-      <c r="E19" s="31" t="n">
+        <v>16606.37963875</v>
+      </c>
+      <c r="E19" s="30" t="n">
         <f aca="false">E8-E13-E15-E17</f>
-        <v>16618.9880928785</v>
-      </c>
-      <c r="F19" s="31" t="n">
+        <v>16662.6219143506</v>
+      </c>
+      <c r="F19" s="30" t="n">
         <f aca="false">F8-F13-F15-F17</f>
-        <v>16635.2301285066</v>
-      </c>
-      <c r="G19" s="31" t="n">
+        <v>16686.6717354683</v>
+      </c>
+      <c r="G19" s="30" t="n">
         <f aca="false">G8-G13-G15-G17</f>
-        <v>16623.5807616318</v>
-      </c>
-      <c r="H19" s="31" t="n">
+        <v>16683.5174882495</v>
+      </c>
+      <c r="H19" s="30" t="n">
         <f aca="false">H8-H13-H15-H17</f>
-        <v>16585.0954259875</v>
-      </c>
-      <c r="I19" s="31" t="n">
+        <v>16654.2672597404</v>
+      </c>
+      <c r="I19" s="30" t="n">
         <f aca="false">I8-I13-I15-I17</f>
-        <v>16520.518579846</v>
-      </c>
-      <c r="J19" s="31" t="n">
+        <v>16599.7243520634</v>
+      </c>
+      <c r="J19" s="30" t="n">
         <f aca="false">J8-J13-J15-J17</f>
-        <v>16430.4946464147</v>
+        <v>16520.596748068</v>
       </c>
     </row>
   </sheetData>
@@ -5484,7 +5457,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:J28"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
@@ -5546,27 +5519,27 @@
       </c>
       <c r="E5" s="19" t="n">
         <f aca="false">D13</f>
-        <v>265.448217480469</v>
+        <v>262.254692109375</v>
       </c>
       <c r="F5" s="19" t="n">
         <f aca="false">E13</f>
-        <v>303.819344984067</v>
+        <v>299.088151403601</v>
       </c>
       <c r="G5" s="19" t="n">
         <f aca="false">F13</f>
-        <v>330.402936332321</v>
+        <v>324.111678709486</v>
       </c>
       <c r="H5" s="19" t="n">
         <f aca="false">G13</f>
-        <v>356.743671725486</v>
+        <v>348.762075164477</v>
       </c>
       <c r="I5" s="19" t="n">
         <f aca="false">H13</f>
-        <v>383.624838526098</v>
+        <v>373.806013193608</v>
       </c>
       <c r="J5" s="19" t="n">
         <f aca="false">I13</f>
-        <v>411.204128818474</v>
+        <v>399.389113225683</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5575,31 +5548,31 @@
       </c>
       <c r="D6" s="19" t="n">
         <f aca="false">'Operating Model'!D19</f>
-        <v>16569.8822059375</v>
+        <v>16606.37963875</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">'Operating Model'!E19</f>
-        <v>16618.9880928785</v>
+        <v>16662.6219143506</v>
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">'Operating Model'!F19</f>
-        <v>16635.2301285066</v>
+        <v>16686.6717354683</v>
       </c>
       <c r="G6" s="19" t="n">
         <f aca="false">'Operating Model'!G19</f>
-        <v>16623.5807616318</v>
+        <v>16683.5174882495</v>
       </c>
       <c r="H6" s="19" t="n">
         <f aca="false">'Operating Model'!H19</f>
-        <v>16585.0954259875</v>
+        <v>16654.2672597404</v>
       </c>
       <c r="I6" s="19" t="n">
         <f aca="false">'Operating Model'!I19</f>
-        <v>16520.518579846</v>
+        <v>16599.7243520634</v>
       </c>
       <c r="J6" s="19" t="n">
         <f aca="false">'Operating Model'!J19</f>
-        <v>16430.4946464147</v>
+        <v>16520.596748068</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5608,31 +5581,31 @@
       </c>
       <c r="D7" s="19" t="n">
         <f aca="false">SUM(D15,D18,D23)</f>
-        <v>11649.98055375</v>
+        <v>11795.970285</v>
       </c>
       <c r="E7" s="19" t="n">
         <f aca="false">SUM(E15,E18,E23)</f>
-        <v>11330.5966181139</v>
+        <v>11505.1319040023</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">SUM(F15,F18,F23)</f>
-        <v>10959.8723196736</v>
+        <v>11165.6387475201</v>
       </c>
       <c r="G7" s="19" t="n">
         <f aca="false">SUM(G15,G18,G23)</f>
-        <v>10553.3547778563</v>
+        <v>10793.1016843274</v>
       </c>
       <c r="H7" s="19" t="n">
         <f aca="false">SUM(H15,H18,H23)</f>
-        <v>10111.1115087954</v>
+        <v>10387.7988438072</v>
       </c>
       <c r="I7" s="19" t="n">
         <f aca="false">SUM(I15,I18,I23)</f>
-        <v>9632.14718477652</v>
+        <v>9948.97027364607</v>
       </c>
       <c r="J7" s="19" t="n">
         <f aca="false">SUM(J15,J18,J23)</f>
-        <v>9115.24027114113</v>
+        <v>9475.64867775454</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5641,31 +5614,31 @@
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">D19</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="E8" s="19" t="n">
         <f aca="false">E19</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="F8" s="19" t="n">
         <f aca="false">F19</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="G8" s="19" t="n">
         <f aca="false">G19</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="H8" s="19" t="n">
         <f aca="false">H19</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="I8" s="19" t="n">
         <f aca="false">I19</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="J8" s="19" t="n">
         <f aca="false">J19</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5674,31 +5647,31 @@
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">D5+D6-D7-D8</f>
-        <v>3947.1714796875</v>
+        <v>3896.07507375</v>
       </c>
       <c r="E9" s="19" t="n">
         <f aca="false">E5+E6-E7-E8</f>
-        <v>4561.10951974507</v>
+        <v>4485.41042245762</v>
       </c>
       <c r="F9" s="19" t="n">
         <f aca="false">F5+F6-F7-F8</f>
-        <v>4986.44698131714</v>
+        <v>4885.78685935178</v>
       </c>
       <c r="G9" s="19" t="n">
         <f aca="false">G5+G6-G7-G8</f>
-        <v>5407.89874760778</v>
+        <v>5280.19320263163</v>
       </c>
       <c r="H9" s="19" t="n">
         <f aca="false">H5+H6-H7-H8</f>
-        <v>5837.99741641757</v>
+        <v>5680.89621109773</v>
       </c>
       <c r="I9" s="19" t="n">
         <f aca="false">I5+I6-I7-I8</f>
-        <v>6279.26606109558</v>
+        <v>6090.22581161093</v>
       </c>
       <c r="J9" s="19" t="n">
         <f aca="false">J5+J6-J7-J8</f>
-        <v>6733.72833159203</v>
+        <v>6510.00290353918</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5740,31 +5713,31 @@
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">MIN(MAX(0,D17-D19),MAX(0,D9+D10-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>2945.37860976562</v>
+        <v>2907.0563053125</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">MIN(MAX(0,E17-E19),MAX(0,E9+E10-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>3405.8321398088</v>
+        <v>3349.05781684321</v>
       </c>
       <c r="F11" s="19" t="n">
         <f aca="false">MIN(MAX(0,F17-F19),MAX(0,F9+F10-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>3724.83523598785</v>
+        <v>3649.34014451383</v>
       </c>
       <c r="G11" s="19" t="n">
         <f aca="false">MIN(MAX(0,G17-G19),MAX(0,G9+G10-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>4040.92406070584</v>
+        <v>3945.14490197372</v>
       </c>
       <c r="H11" s="19" t="n">
         <f aca="false">MIN(MAX(0,H17-H19),MAX(0,H9+H10-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>4363.49806231318</v>
+        <v>4245.67215832329</v>
       </c>
       <c r="I11" s="19" t="n">
         <f aca="false">MIN(MAX(0,I17-I19),MAX(0,I9+I10-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>4694.44954582169</v>
+        <v>4552.6693587082</v>
       </c>
       <c r="J11" s="19" t="n">
         <f aca="false">MIN(MAX(0,J17-J19),MAX(0,J9+J10-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>5035.29624869402</v>
+        <v>4867.50217765439</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5773,68 +5746,68 @@
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">MIN(MAX(0,D22+D24),MAX(0,D9+D10-D11-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>736.344652441406</v>
+        <v>726.764076328124</v>
       </c>
       <c r="E12" s="19" t="n">
         <f aca="false">MIN(MAX(0,E22+E24),MAX(0,E9+E10-E11-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>851.458034952201</v>
+        <v>837.264454210804</v>
       </c>
       <c r="F12" s="19" t="n">
         <f aca="false">MIN(MAX(0,F22+F24),MAX(0,F9+F10-F11-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>931.208808996963</v>
+        <v>912.335036128458</v>
       </c>
       <c r="G12" s="19" t="n">
         <f aca="false">MIN(MAX(0,G22+G24),MAX(0,G9+G10-G11-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>1010.23101517646</v>
+        <v>986.28622549343</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">MIN(MAX(0,H22+H24),MAX(0,H9+H10-H11-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>1090.87451557829</v>
+        <v>1061.41803958082</v>
       </c>
       <c r="I12" s="19" t="n">
         <f aca="false">MIN(MAX(0,I22+I24),MAX(0,I9+I10-I11-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>1173.61238645542</v>
+        <v>1138.16733967705</v>
       </c>
       <c r="J12" s="19" t="n">
         <f aca="false">MIN(MAX(0,J22+J24),MAX(0,J9+J10-J11-Assumptions!$E$16)*Assumptions!$E$25)</f>
-        <v>1258.82406217351</v>
+        <v>1216.8755444136</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="29" t="s">
         <v>212</v>
       </c>
-      <c r="C13" s="31" t="n">
+      <c r="C13" s="30" t="n">
         <f aca="false">C5</f>
         <v>20</v>
       </c>
-      <c r="D13" s="31" t="n">
+      <c r="D13" s="30" t="n">
         <f aca="false">D9+D10-D11-D12</f>
-        <v>265.448217480469</v>
-      </c>
-      <c r="E13" s="31" t="n">
+        <v>262.254692109375</v>
+      </c>
+      <c r="E13" s="30" t="n">
         <f aca="false">E9+E10-E11-E12</f>
-        <v>303.819344984067</v>
-      </c>
-      <c r="F13" s="31" t="n">
+        <v>299.088151403601</v>
+      </c>
+      <c r="F13" s="30" t="n">
         <f aca="false">F9+F10-F11-F12</f>
-        <v>330.402936332321</v>
-      </c>
-      <c r="G13" s="31" t="n">
+        <v>324.111678709486</v>
+      </c>
+      <c r="G13" s="30" t="n">
         <f aca="false">G9+G10-G11-G12</f>
-        <v>356.743671725486</v>
-      </c>
-      <c r="H13" s="31" t="n">
+        <v>348.762075164477</v>
+      </c>
+      <c r="H13" s="30" t="n">
         <f aca="false">H9+H10-H11-H12</f>
-        <v>383.624838526098</v>
-      </c>
-      <c r="I13" s="31" t="n">
+        <v>373.806013193608</v>
+      </c>
+      <c r="I13" s="30" t="n">
         <f aca="false">I9+I10-I11-I12</f>
-        <v>411.204128818474</v>
-      </c>
-      <c r="J13" s="31" t="n">
+        <v>399.389113225683</v>
+      </c>
+      <c r="J13" s="30" t="n">
         <f aca="false">J9+J10-J11-J12</f>
-        <v>439.608020724502</v>
+        <v>425.625181471199</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5950,35 +5923,35 @@
       </c>
       <c r="C17" s="19" t="n">
         <f aca="false">'Sources &amp; Uses'!F6</f>
-        <v>99273.01725</v>
+        <v>93433.428</v>
       </c>
       <c r="D17" s="19" t="n">
         <f aca="false">C21</f>
-        <v>99273.01725</v>
+        <v>93433.428</v>
       </c>
       <c r="E17" s="19" t="n">
         <f aca="false">D21</f>
-        <v>95334.9084677344</v>
+        <v>89592.0374146875</v>
       </c>
       <c r="F17" s="19" t="n">
         <f aca="false">E21</f>
-        <v>90936.3461554256</v>
+        <v>85308.6453178443</v>
       </c>
       <c r="G17" s="19" t="n">
         <f aca="false">F21</f>
-        <v>86218.7807469377</v>
+        <v>80724.9708933305</v>
       </c>
       <c r="H17" s="19" t="n">
         <f aca="false">G21</f>
-        <v>81185.1265137319</v>
+        <v>75845.4917113568</v>
       </c>
       <c r="I17" s="19" t="n">
         <f aca="false">H21</f>
-        <v>75828.8982789187</v>
+        <v>70665.4852730335</v>
       </c>
       <c r="J17" s="19" t="n">
         <f aca="false">I21</f>
-        <v>70141.718560597</v>
+        <v>65178.4816343253</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5987,31 +5960,31 @@
       </c>
       <c r="D18" s="19" t="n">
         <f aca="false">D17*Assumptions!$E$20</f>
-        <v>8438.20646625</v>
+        <v>7941.84138</v>
       </c>
       <c r="E18" s="19" t="n">
         <f aca="false">E17*Assumptions!$E$20</f>
-        <v>8103.46721975742</v>
+        <v>7615.32318024844</v>
       </c>
       <c r="F18" s="19" t="n">
         <f aca="false">F17*Assumptions!$E$20</f>
-        <v>7729.58942321118</v>
+        <v>7251.23485201677</v>
       </c>
       <c r="G18" s="19" t="n">
         <f aca="false">G17*Assumptions!$E$20</f>
-        <v>7328.59636348971</v>
+        <v>6861.62252593309</v>
       </c>
       <c r="H18" s="19" t="n">
         <f aca="false">H17*Assumptions!$E$20</f>
-        <v>6900.73575366721</v>
+        <v>6446.86679546533</v>
       </c>
       <c r="I18" s="19" t="n">
         <f aca="false">I17*Assumptions!$E$20</f>
-        <v>6445.45635370809</v>
+        <v>6006.56624820785</v>
       </c>
       <c r="J18" s="19" t="n">
         <f aca="false">J17*Assumptions!$E$20</f>
-        <v>5962.04607765075</v>
+        <v>5540.17093891765</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6020,68 +5993,68 @@
       </c>
       <c r="D19" s="19" t="n">
         <f aca="false">MIN(D17,'Sources &amp; Uses'!$F$6*Assumptions!$E$21)</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="E19" s="19" t="n">
         <f aca="false">MIN(E17,'Sources &amp; Uses'!$F$6*Assumptions!$E$21)</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="F19" s="19" t="n">
         <f aca="false">MIN(F17,'Sources &amp; Uses'!$F$6*Assumptions!$E$21)</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="G19" s="19" t="n">
         <f aca="false">MIN(G17,'Sources &amp; Uses'!$F$6*Assumptions!$E$21)</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="H19" s="19" t="n">
         <f aca="false">MIN(H17,'Sources &amp; Uses'!$F$6*Assumptions!$E$21)</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="I19" s="19" t="n">
         <f aca="false">MIN(I17,'Sources &amp; Uses'!$F$6*Assumptions!$E$21)</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
       <c r="J19" s="19" t="n">
         <f aca="false">MIN(J17,'Sources &amp; Uses'!$F$6*Assumptions!$E$21)</f>
-        <v>992.7301725</v>
+        <v>934.33428</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="29" t="s">
         <v>219</v>
       </c>
-      <c r="C20" s="31" t="n">
+      <c r="C20" s="30" t="n">
         <f aca="false">'Sources &amp; Uses'!F7</f>
-        <v>29197.94625</v>
-      </c>
-      <c r="D20" s="31" t="n">
+        <v>35037.5355</v>
+      </c>
+      <c r="D20" s="30" t="n">
         <f aca="false">D11</f>
-        <v>2945.37860976562</v>
-      </c>
-      <c r="E20" s="31" t="n">
+        <v>2907.0563053125</v>
+      </c>
+      <c r="E20" s="30" t="n">
         <f aca="false">E11</f>
-        <v>3405.8321398088</v>
-      </c>
-      <c r="F20" s="31" t="n">
+        <v>3349.05781684321</v>
+      </c>
+      <c r="F20" s="30" t="n">
         <f aca="false">F11</f>
-        <v>3724.83523598785</v>
-      </c>
-      <c r="G20" s="31" t="n">
+        <v>3649.34014451383</v>
+      </c>
+      <c r="G20" s="30" t="n">
         <f aca="false">G11</f>
-        <v>4040.92406070584</v>
-      </c>
-      <c r="H20" s="31" t="n">
+        <v>3945.14490197372</v>
+      </c>
+      <c r="H20" s="30" t="n">
         <f aca="false">H11</f>
-        <v>4363.49806231318</v>
-      </c>
-      <c r="I20" s="31" t="n">
+        <v>4245.67215832329</v>
+      </c>
+      <c r="I20" s="30" t="n">
         <f aca="false">I11</f>
-        <v>4694.44954582169</v>
-      </c>
-      <c r="J20" s="31" t="n">
+        <v>4552.6693587082</v>
+      </c>
+      <c r="J20" s="30" t="n">
         <f aca="false">J11</f>
-        <v>5035.29624869402</v>
+        <v>4867.50217765439</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6090,35 +6063,35 @@
       </c>
       <c r="C21" s="19" t="n">
         <f aca="false">C17</f>
-        <v>99273.01725</v>
+        <v>93433.428</v>
       </c>
       <c r="D21" s="19" t="n">
         <f aca="false">MAX(0,D17-D19-D20)</f>
-        <v>95334.9084677344</v>
+        <v>89592.0374146875</v>
       </c>
       <c r="E21" s="19" t="n">
         <f aca="false">MAX(0,E17-E19-E20)</f>
-        <v>90936.3461554256</v>
+        <v>85308.6453178443</v>
       </c>
       <c r="F21" s="19" t="n">
         <f aca="false">MAX(0,F17-F19-F20)</f>
-        <v>86218.7807469377</v>
+        <v>80724.9708933305</v>
       </c>
       <c r="G21" s="19" t="n">
         <f aca="false">MAX(0,G17-G19-G20)</f>
-        <v>81185.1265137319</v>
+        <v>75845.4917113568</v>
       </c>
       <c r="H21" s="19" t="n">
         <f aca="false">MAX(0,H17-H19-H20)</f>
-        <v>75828.8982789187</v>
+        <v>70665.4852730335</v>
       </c>
       <c r="I21" s="19" t="n">
         <f aca="false">MAX(0,I17-I19-I20)</f>
-        <v>70141.718560597</v>
+        <v>65178.4816343253</v>
       </c>
       <c r="J21" s="19" t="n">
         <f aca="false">MAX(0,J17-J19-J20)</f>
-        <v>64113.692139403</v>
+        <v>59376.6451766709</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6127,35 +6100,35 @@
       </c>
       <c r="C22" s="19" t="n">
         <f aca="false">'Sources &amp; Uses'!F7</f>
-        <v>29197.94625</v>
+        <v>35037.5355</v>
       </c>
       <c r="D22" s="19" t="n">
         <f aca="false">C26</f>
-        <v>29197.94625</v>
+        <v>35037.5355</v>
       </c>
       <c r="E22" s="19" t="n">
         <f aca="false">D26</f>
-        <v>29337.5399850586</v>
+        <v>35361.8974886719</v>
       </c>
       <c r="F22" s="19" t="n">
         <f aca="false">E26</f>
-        <v>29366.2081496582</v>
+        <v>35585.4899591212</v>
       </c>
       <c r="G22" s="19" t="n">
         <f aca="false">F26</f>
-        <v>29315.9855851509</v>
+        <v>35740.7196217664</v>
       </c>
       <c r="H22" s="19" t="n">
         <f aca="false">G26</f>
-        <v>29185.234137529</v>
+        <v>35826.654984926</v>
       </c>
       <c r="I22" s="19" t="n">
         <f aca="false">H26</f>
-        <v>28969.9166460766</v>
+        <v>35840.0365948929</v>
       </c>
       <c r="J22" s="19" t="n">
         <f aca="false">I26</f>
-        <v>28665.4017590035</v>
+        <v>35777.0703530627</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6164,139 +6137,139 @@
       </c>
       <c r="D23" s="19" t="n">
         <f aca="false">D22*Assumptions!$E$23</f>
-        <v>3211.7740875</v>
+        <v>3854.128905</v>
       </c>
       <c r="E23" s="19" t="n">
         <f aca="false">E22*Assumptions!$E$23</f>
-        <v>3227.12939835645</v>
+        <v>3889.80872375391</v>
       </c>
       <c r="F23" s="19" t="n">
         <f aca="false">F22*Assumptions!$E$23</f>
-        <v>3230.2828964624</v>
+        <v>3914.40389550333</v>
       </c>
       <c r="G23" s="19" t="n">
         <f aca="false">G22*Assumptions!$E$23</f>
-        <v>3224.7584143666</v>
+        <v>3931.4791583943</v>
       </c>
       <c r="H23" s="19" t="n">
         <f aca="false">H22*Assumptions!$E$23</f>
-        <v>3210.37575512819</v>
+        <v>3940.93204834186</v>
       </c>
       <c r="I23" s="19" t="n">
         <f aca="false">I22*Assumptions!$E$23</f>
-        <v>3186.69083106842</v>
+        <v>3942.40402543822</v>
       </c>
       <c r="J23" s="19" t="n">
         <f aca="false">J22*Assumptions!$E$23</f>
-        <v>3153.19419349038</v>
+        <v>3935.47773883689</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="30" t="s">
+      <c r="B24" s="29" t="s">
         <v>223</v>
       </c>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31" t="n">
+      <c r="C24" s="30"/>
+      <c r="D24" s="30" t="n">
         <f aca="false">D22*Assumptions!$E$24</f>
-        <v>875.9383875</v>
-      </c>
-      <c r="E24" s="31" t="n">
+        <v>1051.126065</v>
+      </c>
+      <c r="E24" s="30" t="n">
         <f aca="false">E22*Assumptions!$E$24</f>
-        <v>880.126199551758</v>
-      </c>
-      <c r="F24" s="31" t="n">
+        <v>1060.85692466016</v>
+      </c>
+      <c r="F24" s="30" t="n">
         <f aca="false">F22*Assumptions!$E$24</f>
-        <v>880.986244489744</v>
-      </c>
-      <c r="G24" s="31" t="n">
+        <v>1067.56469877364</v>
+      </c>
+      <c r="G24" s="30" t="n">
         <f aca="false">G22*Assumptions!$E$24</f>
-        <v>879.479567554528</v>
-      </c>
-      <c r="H24" s="31" t="n">
+        <v>1072.22158865299</v>
+      </c>
+      <c r="H24" s="30" t="n">
         <f aca="false">H22*Assumptions!$E$24</f>
-        <v>875.55702412587</v>
-      </c>
-      <c r="I24" s="31" t="n">
+        <v>1074.79964954778</v>
+      </c>
+      <c r="I24" s="30" t="n">
         <f aca="false">I22*Assumptions!$E$24</f>
-        <v>869.097499382297</v>
-      </c>
-      <c r="J24" s="31" t="n">
+        <v>1075.20109784679</v>
+      </c>
+      <c r="J24" s="30" t="n">
         <f aca="false">J22*Assumptions!$E$24</f>
-        <v>859.962052770104</v>
+        <v>1073.31211059188</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="29" t="s">
         <v>224</v>
       </c>
-      <c r="C25" s="31" t="n">
+      <c r="C25" s="30" t="n">
         <f aca="false">SUM(C16,C20,C13)</f>
-        <v>29217.94625</v>
-      </c>
-      <c r="D25" s="31" t="n">
+        <v>35057.5355</v>
+      </c>
+      <c r="D25" s="30" t="n">
         <f aca="false">D12</f>
-        <v>736.344652441406</v>
-      </c>
-      <c r="E25" s="31" t="n">
+        <v>726.764076328124</v>
+      </c>
+      <c r="E25" s="30" t="n">
         <f aca="false">E12</f>
-        <v>851.458034952201</v>
-      </c>
-      <c r="F25" s="31" t="n">
+        <v>837.264454210804</v>
+      </c>
+      <c r="F25" s="30" t="n">
         <f aca="false">F12</f>
-        <v>931.208808996963</v>
-      </c>
-      <c r="G25" s="31" t="n">
+        <v>912.335036128458</v>
+      </c>
+      <c r="G25" s="30" t="n">
         <f aca="false">G12</f>
-        <v>1010.23101517646</v>
-      </c>
-      <c r="H25" s="31" t="n">
+        <v>986.28622549343</v>
+      </c>
+      <c r="H25" s="30" t="n">
         <f aca="false">H12</f>
-        <v>1090.87451557829</v>
-      </c>
-      <c r="I25" s="31" t="n">
+        <v>1061.41803958082</v>
+      </c>
+      <c r="I25" s="30" t="n">
         <f aca="false">I12</f>
-        <v>1173.61238645542</v>
-      </c>
-      <c r="J25" s="31" t="n">
+        <v>1138.16733967705</v>
+      </c>
+      <c r="J25" s="30" t="n">
         <f aca="false">J12</f>
-        <v>1258.82406217351</v>
+        <v>1216.8755444136</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="30" t="s">
+      <c r="B26" s="29" t="s">
         <v>225</v>
       </c>
-      <c r="C26" s="31" t="n">
+      <c r="C26" s="30" t="n">
         <f aca="false">C22</f>
-        <v>29197.94625</v>
-      </c>
-      <c r="D26" s="31" t="n">
+        <v>35037.5355</v>
+      </c>
+      <c r="D26" s="30" t="n">
         <f aca="false">MAX(0,D22+D24-D25)</f>
-        <v>29337.5399850586</v>
-      </c>
-      <c r="E26" s="31" t="n">
+        <v>35361.8974886719</v>
+      </c>
+      <c r="E26" s="30" t="n">
         <f aca="false">MAX(0,E22+E24-E25)</f>
-        <v>29366.2081496582</v>
-      </c>
-      <c r="F26" s="31" t="n">
+        <v>35585.4899591212</v>
+      </c>
+      <c r="F26" s="30" t="n">
         <f aca="false">MAX(0,F22+F24-F25)</f>
-        <v>29315.9855851509</v>
-      </c>
-      <c r="G26" s="31" t="n">
+        <v>35740.7196217664</v>
+      </c>
+      <c r="G26" s="30" t="n">
         <f aca="false">MAX(0,G22+G24-G25)</f>
-        <v>29185.234137529</v>
-      </c>
-      <c r="H26" s="31" t="n">
+        <v>35826.654984926</v>
+      </c>
+      <c r="H26" s="30" t="n">
         <f aca="false">MAX(0,H22+H24-H25)</f>
-        <v>28969.9166460766</v>
-      </c>
-      <c r="I26" s="31" t="n">
+        <v>35840.0365948929</v>
+      </c>
+      <c r="I26" s="30" t="n">
         <f aca="false">MAX(0,I22+I24-I25)</f>
-        <v>28665.4017590035</v>
-      </c>
-      <c r="J26" s="31" t="n">
+        <v>35777.0703530627</v>
+      </c>
+      <c r="J26" s="30" t="n">
         <f aca="false">MAX(0,J22+J24-J25)</f>
-        <v>28266.5397496001</v>
+        <v>35633.5069192409</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6309,31 +6282,31 @@
       </c>
       <c r="D27" s="19" t="n">
         <f aca="false">SUM(D16,D21,D26)</f>
-        <v>124672.448452793</v>
+        <v>124953.934903359</v>
       </c>
       <c r="E27" s="19" t="n">
         <f aca="false">SUM(E16,E21,E26)</f>
-        <v>120302.554305084</v>
+        <v>120894.135276966</v>
       </c>
       <c r="F27" s="19" t="n">
         <f aca="false">SUM(F16,F21,F26)</f>
-        <v>115534.766332089</v>
+        <v>116465.690515097</v>
       </c>
       <c r="G27" s="19" t="n">
         <f aca="false">SUM(G16,G21,G26)</f>
-        <v>110370.360651261</v>
+        <v>111672.146696283</v>
       </c>
       <c r="H27" s="19" t="n">
         <f aca="false">SUM(H16,H21,H26)</f>
-        <v>104798.814924995</v>
+        <v>106505.521867926</v>
       </c>
       <c r="I27" s="19" t="n">
         <f aca="false">SUM(I16,I21,I26)</f>
-        <v>98807.1203196005</v>
+        <v>100955.551987388</v>
       </c>
       <c r="J27" s="19" t="n">
         <f aca="false">SUM(J16,J21,J26)</f>
-        <v>92380.2318890031</v>
+        <v>95010.1520959118</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6346,31 +6319,31 @@
       </c>
       <c r="D28" s="19" t="n">
         <f aca="false">D27-D13</f>
-        <v>124407.000235313</v>
+        <v>124691.68021125</v>
       </c>
       <c r="E28" s="19" t="n">
         <f aca="false">E27-E13</f>
-        <v>119998.7349601</v>
+        <v>120595.047125562</v>
       </c>
       <c r="F28" s="19" t="n">
         <f aca="false">F27-F13</f>
-        <v>115204.363395756</v>
+        <v>116141.578836387</v>
       </c>
       <c r="G28" s="19" t="n">
         <f aca="false">G27-G13</f>
-        <v>110013.616979535</v>
+        <v>111323.384621118</v>
       </c>
       <c r="H28" s="19" t="n">
         <f aca="false">H27-H13</f>
-        <v>104415.190086469</v>
+        <v>106131.715854733</v>
       </c>
       <c r="I28" s="19" t="n">
         <f aca="false">I27-I13</f>
-        <v>98395.916190782</v>
+        <v>100556.162874162</v>
       </c>
       <c r="J28" s="19" t="n">
         <f aca="false">J27-J13</f>
-        <v>91940.6238682786</v>
+        <v>94584.5269144406</v>
       </c>
     </row>
   </sheetData>
@@ -6393,7 +6366,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:I13"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
@@ -6442,64 +6415,64 @@
       <c r="B5" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="26" t="n">
         <f aca="false">IFERROR('Debt Schedule'!D25/'Operating Model'!D8,0)</f>
-        <v>0.031470341454065</v>
-      </c>
-      <c r="D5" s="27" t="n">
+        <v>0.0310608810191831</v>
+      </c>
+      <c r="D5" s="26" t="n">
         <f aca="false">IFERROR('Debt Schedule'!E25/'Operating Model'!E8,0)</f>
-        <v>0.0363648092872103</v>
-      </c>
-      <c r="E5" s="27" t="n">
+        <v>0.0357586175131289</v>
+      </c>
+      <c r="E5" s="26" t="n">
         <f aca="false">IFERROR('Debt Schedule'!F25/'Operating Model'!F8,0)</f>
-        <v>0.0397806367317733</v>
-      </c>
-      <c r="F5" s="27" t="n">
+        <v>0.0389743613883853</v>
+      </c>
+      <c r="F5" s="26" t="n">
         <f aca="false">IFERROR('Debt Schedule'!G25/'Operating Model'!G8,0)</f>
-        <v>0.0432052772705459</v>
-      </c>
-      <c r="G5" s="27" t="n">
+        <v>0.0421812132080706</v>
+      </c>
+      <c r="G5" s="26" t="n">
         <f aca="false">IFERROR('Debt Schedule'!H25/'Operating Model'!H8,0)</f>
-        <v>0.046746086843912</v>
-      </c>
-      <c r="H5" s="27" t="n">
+        <v>0.0454838197678832</v>
+      </c>
+      <c r="H5" s="26" t="n">
         <f aca="false">IFERROR('Debt Schedule'!I25/'Operating Model'!I8,0)</f>
-        <v>0.0504303901683732</v>
-      </c>
-      <c r="I5" s="27" t="n">
+        <v>0.048907308477008</v>
+      </c>
+      <c r="I5" s="26" t="n">
         <f aca="false">IFERROR('Debt Schedule'!J25/'Operating Model'!J8,0)</f>
-        <v>0.054281793146728</v>
+        <v>0.052472929754076</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="26" t="n">
         <f aca="false">Assumptions!$E$26</f>
         <v>7</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="26" t="n">
         <f aca="false">Assumptions!$E$26</f>
         <v>7</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="26" t="n">
         <f aca="false">Assumptions!$E$26</f>
         <v>7</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="26" t="n">
         <f aca="false">Assumptions!$E$26</f>
         <v>7</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="26" t="n">
         <f aca="false">Assumptions!$E$26</f>
         <v>7</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="26" t="n">
         <f aca="false">Assumptions!$E$26</f>
         <v>7</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="26" t="n">
         <f aca="false">Assumptions!$E$26</f>
         <v>7</v>
       </c>
@@ -6508,97 +6481,97 @@
       <c r="B7" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="26" t="n">
         <f aca="false">C6-C5</f>
-        <v>6.96852965854594</v>
-      </c>
-      <c r="D7" s="27" t="n">
+        <v>6.96893911898082</v>
+      </c>
+      <c r="D7" s="26" t="n">
         <f aca="false">D6-D5</f>
-        <v>6.96363519071279</v>
-      </c>
-      <c r="E7" s="27" t="n">
+        <v>6.96424138248687</v>
+      </c>
+      <c r="E7" s="26" t="n">
         <f aca="false">E6-E5</f>
-        <v>6.96021936326823</v>
-      </c>
-      <c r="F7" s="27" t="n">
+        <v>6.96102563861161</v>
+      </c>
+      <c r="F7" s="26" t="n">
         <f aca="false">F6-F5</f>
-        <v>6.95679472272945</v>
-      </c>
-      <c r="G7" s="27" t="n">
+        <v>6.95781878679193</v>
+      </c>
+      <c r="G7" s="26" t="n">
         <f aca="false">G6-G5</f>
-        <v>6.95325391315609</v>
-      </c>
-      <c r="H7" s="27" t="n">
+        <v>6.95451618023212</v>
+      </c>
+      <c r="H7" s="26" t="n">
         <f aca="false">H6-H5</f>
-        <v>6.94956960983163</v>
-      </c>
-      <c r="I7" s="27" t="n">
+        <v>6.95109269152299</v>
+      </c>
+      <c r="I7" s="26" t="n">
         <f aca="false">I6-I5</f>
-        <v>6.94571820685327</v>
+        <v>6.94752707024592</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="26" t="n">
         <f aca="false">IFERROR('Operating Model'!D8/'Debt Schedule'!D7,0)</f>
-        <v>2.00841974216587</v>
-      </c>
-      <c r="D8" s="27" t="n">
+        <v>1.98356306218857</v>
+      </c>
+      <c r="D8" s="26" t="n">
         <f aca="false">IFERROR('Operating Model'!E8/'Debt Schedule'!E7,0)</f>
-        <v>2.06647024084047</v>
-      </c>
-      <c r="E8" s="27" t="n">
+        <v>2.03512144994659</v>
+      </c>
+      <c r="E8" s="26" t="n">
         <f aca="false">IFERROR('Operating Model'!F8/'Debt Schedule'!F7,0)</f>
-        <v>2.13584558186835</v>
-      </c>
-      <c r="F8" s="27" t="n">
+        <v>2.09648506468249</v>
+      </c>
+      <c r="F8" s="26" t="n">
         <f aca="false">IFERROR('Operating Model'!G8/'Debt Schedule'!G7,0)</f>
-        <v>2.21561023559757</v>
-      </c>
-      <c r="G8" s="27" t="n">
+        <v>2.16639493906224</v>
+      </c>
+      <c r="G8" s="26" t="n">
         <f aca="false">IFERROR('Operating Model'!H8/'Debt Schedule'!H7,0)</f>
-        <v>2.30797252550207</v>
-      </c>
-      <c r="H8" s="27" t="n">
+        <v>2.24649783033677</v>
+      </c>
+      <c r="H8" s="26" t="n">
         <f aca="false">IFERROR('Operating Model'!I8/'Debt Schedule'!I7,0)</f>
-        <v>2.41606851580647</v>
-      </c>
-      <c r="I8" s="27" t="n">
+        <v>2.3391292679201</v>
+      </c>
+      <c r="I8" s="26" t="n">
         <f aca="false">IFERROR('Operating Model'!J8/'Debt Schedule'!J7,0)</f>
-        <v>2.54415009379848</v>
+        <v>2.44738277868644</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="26" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>1.75</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="26" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>1.75</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="26" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>1.75</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="26" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>1.75</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="26" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>1.75</v>
       </c>
-      <c r="H9" s="27" t="n">
+      <c r="H9" s="26" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>1.75</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="26" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>1.75</v>
       </c>
@@ -6607,33 +6580,33 @@
       <c r="B10" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="26" t="n">
         <f aca="false">C8-C9</f>
-        <v>0.258419742165872</v>
-      </c>
-      <c r="D10" s="27" t="n">
+        <v>0.233563062188571</v>
+      </c>
+      <c r="D10" s="26" t="n">
         <f aca="false">D8-D9</f>
-        <v>0.316470240840472</v>
-      </c>
-      <c r="E10" s="27" t="n">
+        <v>0.285121449946588</v>
+      </c>
+      <c r="E10" s="26" t="n">
         <f aca="false">E8-E9</f>
-        <v>0.385845581868348</v>
-      </c>
-      <c r="F10" s="27" t="n">
+        <v>0.34648506468249</v>
+      </c>
+      <c r="F10" s="26" t="n">
         <f aca="false">F8-F9</f>
-        <v>0.465610235597571</v>
-      </c>
-      <c r="G10" s="27" t="n">
+        <v>0.416394939062236</v>
+      </c>
+      <c r="G10" s="26" t="n">
         <f aca="false">G8-G9</f>
-        <v>0.557972525502074</v>
-      </c>
-      <c r="H10" s="27" t="n">
+        <v>0.496497830336767</v>
+      </c>
+      <c r="H10" s="26" t="n">
         <f aca="false">H8-H9</f>
-        <v>0.666068515806475</v>
-      </c>
-      <c r="I10" s="27" t="n">
+        <v>0.589129267920095</v>
+      </c>
+      <c r="I10" s="26" t="n">
         <f aca="false">I8-I9</f>
-        <v>0.79415009379848</v>
+        <v>0.697382778686439</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6675,31 +6648,31 @@
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">'Debt Schedule'!D13-C11</f>
-        <v>245.448217480469</v>
+        <v>242.254692109375</v>
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">'Debt Schedule'!E13-D11</f>
-        <v>283.819344984067</v>
+        <v>279.088151403601</v>
       </c>
       <c r="E12" s="19" t="n">
         <f aca="false">'Debt Schedule'!F13-E11</f>
-        <v>310.402936332321</v>
+        <v>304.111678709486</v>
       </c>
       <c r="F12" s="19" t="n">
         <f aca="false">'Debt Schedule'!G13-F11</f>
-        <v>336.743671725486</v>
+        <v>328.762075164477</v>
       </c>
       <c r="G12" s="19" t="n">
         <f aca="false">'Debt Schedule'!H13-G11</f>
-        <v>363.624838526098</v>
+        <v>353.806013193608</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">'Debt Schedule'!I13-H11</f>
-        <v>391.204128818474</v>
+        <v>379.389113225683</v>
       </c>
       <c r="I12" s="19" t="n">
         <f aca="false">'Debt Schedule'!J13-I11</f>
-        <v>419.608020724502</v>
+        <v>405.625181471199</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>